<commit_message>
Corrige calculo do saldo disponivel e compromissos por mes
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Exemplo.xlsx
+++ b/ControleFinanceiro_2026_Exemplo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mateus\PROJETOS\meu_controle-financeiro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E903BBC-8243-4959-97A3-1F097C2776AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CC7BFD3-6D52-4A44-BF62-8D6908D916B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4215" yWindow="1530" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1515" windowWidth="21600" windowHeight="11385" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracoes" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="56">
   <si>
     <t>Campo</t>
   </si>
@@ -186,15 +186,22 @@
   </si>
   <si>
     <t xml:space="preserve">Streaming </t>
+  </si>
+  <si>
+    <t>ultima alteraçao</t>
+  </si>
+  <si>
+    <t>valor anterior</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="mm/yyyy"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -244,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -272,6 +279,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -856,29 +864,43 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Planilha3"/>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>52</v>
       </c>
       <c r="B2">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="13">
+        <v>46266</v>
+      </c>
+      <c r="D2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>

</xml_diff>